<commit_message>
calidad: agregar pruebas unitarias en frontend, apuntar app movil a Railway y actualizar plan de pruebas
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totales" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos de Prueba'!$A$12:$N$13</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Casos de Prueba'!$C$1:$N$534</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos de Prueba'!$A$12:$N$13</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -3045,8 +3045,8 @@
   <mergeCells count="70">
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B72:C72"/>
     <mergeCell ref="B25:C25"/>
@@ -3125,7 +3125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X200"/>
+  <dimension ref="A1:X163"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.109375" customWidth="1" style="6" min="1" max="1"/>
@@ -5663,16 +5663,52 @@
       <c r="J69" s="25" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="25" t="n"/>
-      <c r="B70" s="25" t="n"/>
-      <c r="C70" s="25" t="n"/>
-      <c r="D70" s="25" t="n"/>
-      <c r="E70" s="25" t="n"/>
-      <c r="F70" s="25" t="n"/>
-      <c r="G70" s="25" t="n"/>
-      <c r="H70" s="25" t="n"/>
-      <c r="I70" s="25" t="n"/>
-      <c r="J70" s="25" t="n"/>
+      <c r="A70" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B70" s="25" t="inlineStr">
+        <is>
+          <t>Navegación y Menús</t>
+        </is>
+      </c>
+      <c r="C70" s="25" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D70" s="25" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E70" s="25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F70" s="25" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de Barra de Navegación (Navbar)</t>
+        </is>
+      </c>
+      <c r="G70" s="25" t="inlineStr">
+        <is>
+          <t>1. Renderizar Navbar en estado sin sesión.</t>
+        </is>
+      </c>
+      <c r="H70" s="25" t="inlineStr">
+        <is>
+          <t>localStorage vacío, ruta /</t>
+        </is>
+      </c>
+      <c r="I70" s="25" t="inlineStr">
+        <is>
+          <t>Se visualizan enlaces de Quiénes Somos, Contacto, Términos y botones de ingreso.</t>
+        </is>
+      </c>
+      <c r="J70" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="25" t="n"/>
@@ -5681,10 +5717,26 @@
       <c r="D71" s="25" t="n"/>
       <c r="E71" s="25" t="n"/>
       <c r="F71" s="25" t="n"/>
-      <c r="G71" s="25" t="n"/>
-      <c r="H71" s="25" t="n"/>
-      <c r="I71" s="25" t="n"/>
-      <c r="J71" s="25" t="n"/>
+      <c r="G71" s="25" t="inlineStr">
+        <is>
+          <t>2. Renderizar Navbar con sesión activa de Trabajador o Empresa.</t>
+        </is>
+      </c>
+      <c r="H71" s="25" t="inlineStr">
+        <is>
+          <t>localStorage con user_info de TRABAJADOR o EMPRESA</t>
+        </is>
+      </c>
+      <c r="I71" s="25" t="inlineStr">
+        <is>
+          <t>Se visualizan opciones de dashboard específicas por rol y campana de notificaciones.</t>
+        </is>
+      </c>
+      <c r="J71" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="25" t="n"/>
@@ -5693,10 +5745,26 @@
       <c r="D72" s="25" t="n"/>
       <c r="E72" s="25" t="n"/>
       <c r="F72" s="25" t="n"/>
-      <c r="G72" s="25" t="n"/>
-      <c r="H72" s="25" t="n"/>
-      <c r="I72" s="25" t="n"/>
-      <c r="J72" s="25" t="n"/>
+      <c r="G72" s="25" t="inlineStr">
+        <is>
+          <t>3. Ejecutar flujo de cierre de sesión.</t>
+        </is>
+      </c>
+      <c r="H72" s="25" t="inlineStr">
+        <is>
+          <t>Clic en salir y confirmar</t>
+        </is>
+      </c>
+      <c r="I72" s="25" t="inlineStr">
+        <is>
+          <t>Se limpian claves de localStorage y se redirige a /login.</t>
+        </is>
+      </c>
+      <c r="J72" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="25" t="n"/>
@@ -5711,16 +5779,52 @@
       <c r="J73" s="25" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="25" t="n"/>
-      <c r="B74" s="25" t="n"/>
-      <c r="C74" s="25" t="n"/>
-      <c r="D74" s="25" t="n"/>
-      <c r="E74" s="25" t="n"/>
-      <c r="F74" s="25" t="n"/>
-      <c r="G74" s="25" t="n"/>
-      <c r="H74" s="25" t="n"/>
-      <c r="I74" s="25" t="n"/>
-      <c r="J74" s="25" t="n"/>
+      <c r="A74" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B74" s="25" t="inlineStr">
+        <is>
+          <t>Navegación y Menús</t>
+        </is>
+      </c>
+      <c r="C74" s="25" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E74" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="F74" s="25" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de Campana de Notificaciones</t>
+        </is>
+      </c>
+      <c r="G74" s="25" t="inlineStr">
+        <is>
+          <t>1. Renderizar campana con unreadCount &gt; 0.</t>
+        </is>
+      </c>
+      <c r="H74" s="25" t="inlineStr">
+        <is>
+          <t>unreadCount = 1</t>
+        </is>
+      </c>
+      <c r="I74" s="25" t="inlineStr">
+        <is>
+          <t>Se dibuja un círculo rojo con el número de notificaciones no leídas.</t>
+        </is>
+      </c>
+      <c r="J74" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="25" t="n"/>
@@ -5729,10 +5833,26 @@
       <c r="D75" s="25" t="n"/>
       <c r="E75" s="25" t="n"/>
       <c r="F75" s="25" t="n"/>
-      <c r="G75" s="25" t="n"/>
-      <c r="H75" s="25" t="n"/>
-      <c r="I75" s="25" t="n"/>
-      <c r="J75" s="25" t="n"/>
+      <c r="G75" s="25" t="inlineStr">
+        <is>
+          <t>2. Hacer clic en campana y desplegar listado.</t>
+        </is>
+      </c>
+      <c r="H75" s="25" t="inlineStr">
+        <is>
+          <t>Clic en botón campana</t>
+        </is>
+      </c>
+      <c r="I75" s="25" t="inlineStr">
+        <is>
+          <t>Se abre el panel mostrando las notificaciones y botones de Limpiar/Marcar como leída.</t>
+        </is>
+      </c>
+      <c r="J75" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="25" t="n"/>
@@ -5741,10 +5861,26 @@
       <c r="D76" s="25" t="n"/>
       <c r="E76" s="25" t="n"/>
       <c r="F76" s="25" t="n"/>
-      <c r="G76" s="25" t="n"/>
-      <c r="H76" s="25" t="n"/>
-      <c r="I76" s="25" t="n"/>
-      <c r="J76" s="25" t="n"/>
+      <c r="G76" s="25" t="inlineStr">
+        <is>
+          <t>3. Ejecutar limpieza o marcado de lectura.</t>
+        </is>
+      </c>
+      <c r="H76" s="25" t="inlineStr">
+        <is>
+          <t>Clic en Limpiar o en notificación</t>
+        </is>
+      </c>
+      <c r="I76" s="25" t="inlineStr">
+        <is>
+          <t>Se invocan las funciones del contexto clearAll o markAsRead correspondientes.</t>
+        </is>
+      </c>
+      <c r="J76" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="25" t="n"/>
@@ -5759,16 +5895,52 @@
       <c r="J77" s="25" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="25" t="n"/>
-      <c r="B78" s="25" t="n"/>
-      <c r="C78" s="25" t="n"/>
-      <c r="D78" s="25" t="n"/>
-      <c r="E78" s="25" t="n"/>
-      <c r="F78" s="25" t="n"/>
-      <c r="G78" s="25" t="n"/>
-      <c r="H78" s="25" t="n"/>
-      <c r="I78" s="25" t="n"/>
-      <c r="J78" s="25" t="n"/>
+      <c r="A78" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B78" s="25" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C78" s="25" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E78" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F78" s="25" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de Modal de Pago (PaymentGatewayModal)</t>
+        </is>
+      </c>
+      <c r="G78" s="25" t="inlineStr">
+        <is>
+          <t>1. Renderizar modal en transferencia manual sin archivo adjunto.</t>
+        </is>
+      </c>
+      <c r="H78" s="25" t="inlineStr">
+        <is>
+          <t>isOpen = true, file = null</t>
+        </is>
+      </c>
+      <c r="I78" s="25" t="inlineStr">
+        <is>
+          <t>El botón Confirmar Pago está deshabilitado.</t>
+        </is>
+      </c>
+      <c r="J78" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="25" t="n"/>
@@ -5777,10 +5949,26 @@
       <c r="D79" s="25" t="n"/>
       <c r="E79" s="25" t="n"/>
       <c r="F79" s="25" t="n"/>
-      <c r="G79" s="25" t="n"/>
-      <c r="H79" s="25" t="n"/>
-      <c r="I79" s="25" t="n"/>
-      <c r="J79" s="25" t="n"/>
+      <c r="G79" s="25" t="inlineStr">
+        <is>
+          <t>2. Adjuntar comprobante de pago en transferencia manual.</t>
+        </is>
+      </c>
+      <c r="H79" s="25" t="inlineStr">
+        <is>
+          <t>Archivo comprobante.pdf</t>
+        </is>
+      </c>
+      <c r="I79" s="25" t="inlineStr">
+        <is>
+          <t>El botón Confirmar Pago se habilita y al pulsar llama a onSubmit con los datos.</t>
+        </is>
+      </c>
+      <c r="J79" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="25" t="n"/>
@@ -5789,10 +5977,26 @@
       <c r="D80" s="25" t="n"/>
       <c r="E80" s="25" t="n"/>
       <c r="F80" s="25" t="n"/>
-      <c r="G80" s="25" t="n"/>
-      <c r="H80" s="25" t="n"/>
-      <c r="I80" s="25" t="n"/>
-      <c r="J80" s="25" t="n"/>
+      <c r="G80" s="25" t="inlineStr">
+        <is>
+          <t>3. Cambiar a pasarela Webpay Plus y presionar pagar.</t>
+        </is>
+      </c>
+      <c r="H80" s="25" t="inlineStr">
+        <is>
+          <t>Clic en pestaña Webpay y botón pagar</t>
+        </is>
+      </c>
+      <c r="I80" s="25" t="inlineStr">
+        <is>
+          <t>Se invoca la función onPayWithWebpay y el botón muestra estado de carga.</t>
+        </is>
+      </c>
+      <c r="J80" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="25" t="n"/>
@@ -5807,16 +6011,52 @@
       <c r="J81" s="25" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="25" t="n"/>
-      <c r="B82" s="25" t="n"/>
-      <c r="C82" s="25" t="n"/>
-      <c r="D82" s="25" t="n"/>
-      <c r="E82" s="25" t="n"/>
-      <c r="F82" s="25" t="n"/>
-      <c r="G82" s="25" t="n"/>
-      <c r="H82" s="25" t="n"/>
-      <c r="I82" s="25" t="n"/>
-      <c r="J82" s="25" t="n"/>
+      <c r="A82" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B82" s="25" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="C82" s="25" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D82" s="25" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E82" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="F82" s="25" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de Página de Login (page.tsx)</t>
+        </is>
+      </c>
+      <c r="G82" s="25" t="inlineStr">
+        <is>
+          <t>1. Intentar iniciar sesión con campos vacíos.</t>
+        </is>
+      </c>
+      <c r="H82" s="25" t="inlineStr">
+        <is>
+          <t>email = "", password = ""</t>
+        </is>
+      </c>
+      <c r="I82" s="25" t="inlineStr">
+        <is>
+          <t>Se despliegan mensajes locales indicando que los campos son obligatorios.</t>
+        </is>
+      </c>
+      <c r="J82" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="25" t="n"/>
@@ -5825,10 +6065,26 @@
       <c r="D83" s="25" t="n"/>
       <c r="E83" s="25" t="n"/>
       <c r="F83" s="25" t="n"/>
-      <c r="G83" s="25" t="n"/>
-      <c r="H83" s="25" t="n"/>
-      <c r="I83" s="25" t="n"/>
-      <c r="J83" s="25" t="n"/>
+      <c r="G83" s="25" t="inlineStr">
+        <is>
+          <t>2. Iniciar sesión exitosamente mediante API.</t>
+        </is>
+      </c>
+      <c r="H83" s="25" t="inlineStr">
+        <is>
+          <t>Credenciales correctas de Trabajador / Empresa</t>
+        </is>
+      </c>
+      <c r="I83" s="25" t="inlineStr">
+        <is>
+          <t>Guarda auth_token e user_info en localStorage y redirige al perfil correspondiente.</t>
+        </is>
+      </c>
+      <c r="J83" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="25" t="n"/>
@@ -5837,10 +6093,26 @@
       <c r="D84" s="25" t="n"/>
       <c r="E84" s="25" t="n"/>
       <c r="F84" s="25" t="n"/>
-      <c r="G84" s="25" t="n"/>
-      <c r="H84" s="25" t="n"/>
-      <c r="I84" s="25" t="n"/>
-      <c r="J84" s="25" t="n"/>
+      <c r="G84" s="25" t="inlineStr">
+        <is>
+          <t>3. Iniciar sesión con error de credenciales.</t>
+        </is>
+      </c>
+      <c r="H84" s="25" t="inlineStr">
+        <is>
+          <t>Credenciales erróneas</t>
+        </is>
+      </c>
+      <c r="I84" s="25" t="inlineStr">
+        <is>
+          <t>Se despliega el mensaje de error retornado por la API de autenticación.</t>
+        </is>
+      </c>
+      <c r="J84" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="25" t="n"/>
@@ -6142,9 +6414,6 @@
       <c r="I109" s="25" t="n"/>
       <c r="J109" s="25" t="n"/>
     </row>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
     <row r="113" ht="42.6" customHeight="1"/>
     <row r="114">
       <c r="A114" s="25" t="n"/>
@@ -6696,49 +6965,11 @@
       <c r="H163" s="25" t="n"/>
       <c r="I163" s="25" t="n"/>
     </row>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
   </sheetData>
   <autoFilter ref="A12:N13"/>
   <mergeCells count="282">
     <mergeCell ref="F53:F54"/>
     <mergeCell ref="F17:F19"/>
-    <mergeCell ref="L64:L66"/>
     <mergeCell ref="H53:H54"/>
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="E39:E40"/>
@@ -6801,14 +7032,13 @@
     <mergeCell ref="F43:F45"/>
     <mergeCell ref="N41:N42"/>
     <mergeCell ref="H41:H42"/>
-    <mergeCell ref="F64:F66"/>
     <mergeCell ref="A14:A16"/>
     <mergeCell ref="K14:K16"/>
+    <mergeCell ref="B58:B59"/>
     <mergeCell ref="F20:F21"/>
     <mergeCell ref="H49:H50"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="J49:J50"/>
-    <mergeCell ref="B58:B59"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E22:E24"/>
     <mergeCell ref="L58:L59"/>
@@ -6838,7 +7068,6 @@
     <mergeCell ref="E64:E66"/>
     <mergeCell ref="J34:J36"/>
     <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D67:D68"/>
     <mergeCell ref="J28:J30"/>
     <mergeCell ref="B46:B48"/>
     <mergeCell ref="L28:L30"/>
@@ -6904,6 +7133,7 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="L17:L19"/>
     <mergeCell ref="L60:L61"/>
+    <mergeCell ref="E46:E48"/>
     <mergeCell ref="D34:D36"/>
     <mergeCell ref="B43:B45"/>
     <mergeCell ref="N60:N61"/>
@@ -6951,6 +7181,7 @@
     <mergeCell ref="H28:H30"/>
     <mergeCell ref="J37:J38"/>
     <mergeCell ref="J22:J24"/>
+    <mergeCell ref="F64:F66"/>
     <mergeCell ref="L37:L38"/>
     <mergeCell ref="D64:D66"/>
     <mergeCell ref="L22:L24"/>
@@ -6963,7 +7194,6 @@
     <mergeCell ref="F14:F16"/>
     <mergeCell ref="N31:N33"/>
     <mergeCell ref="B39:B40"/>
-    <mergeCell ref="F67:F68"/>
     <mergeCell ref="E25:E27"/>
     <mergeCell ref="B64:B66"/>
     <mergeCell ref="A8:C8"/>
@@ -6988,11 +7218,15 @@
     <mergeCell ref="D17:D19"/>
     <mergeCell ref="D58:D59"/>
     <mergeCell ref="L49:L50"/>
+    <mergeCell ref="D67:D68"/>
     <mergeCell ref="E28:E30"/>
     <mergeCell ref="F58:F59"/>
+    <mergeCell ref="F67:F68"/>
     <mergeCell ref="N49:N50"/>
+    <mergeCell ref="K62:K63"/>
     <mergeCell ref="A62:A63"/>
     <mergeCell ref="C53:C54"/>
+    <mergeCell ref="M62:M63"/>
     <mergeCell ref="E31:E33"/>
     <mergeCell ref="L43:L45"/>
     <mergeCell ref="E53:E54"/>
@@ -7002,21 +7236,19 @@
     <mergeCell ref="M22:M24"/>
     <mergeCell ref="K31:K33"/>
     <mergeCell ref="D51:D52"/>
-    <mergeCell ref="K62:K63"/>
+    <mergeCell ref="L64:L66"/>
     <mergeCell ref="M31:M33"/>
     <mergeCell ref="D60:D61"/>
-    <mergeCell ref="M62:M63"/>
     <mergeCell ref="N51:N52"/>
     <mergeCell ref="F60:F61"/>
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="C37:C38"/>
     <mergeCell ref="B41:B42"/>
     <mergeCell ref="E37:E38"/>
+    <mergeCell ref="C46:C48"/>
     <mergeCell ref="A46:A48"/>
+    <mergeCell ref="M28:M30"/>
     <mergeCell ref="K46:K48"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="M28:M30"/>
-    <mergeCell ref="E46:E48"/>
     <mergeCell ref="N17:N19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7087,7 +7319,7 @@
         </is>
       </c>
       <c r="C11" s="29" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -7097,7 +7329,7 @@
         </is>
       </c>
       <c r="C12" s="29" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
docs: actualizar planilla de casos de prueba excel y agregar analista de testing
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -2829,7 +2829,11 @@
         </is>
       </c>
       <c r="C61" s="140" t="n"/>
-      <c r="D61" s="35" t="n"/>
+      <c r="D61" s="35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="35" t="inlineStr">
@@ -2843,7 +2847,11 @@
         </is>
       </c>
       <c r="C62" s="142" t="n"/>
-      <c r="D62" s="35" t="n"/>
+      <c r="D62" s="35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="inlineStr">
@@ -2857,7 +2865,11 @@
         </is>
       </c>
       <c r="C63" s="80" t="n"/>
-      <c r="D63" s="35" t="n"/>
+      <c r="D63" s="35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="36" t="n"/>
@@ -2913,7 +2925,11 @@
         </is>
       </c>
       <c r="C71" s="140" t="n"/>
-      <c r="D71" s="37" t="n"/>
+      <c r="D71" s="37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="35" t="inlineStr">
@@ -2927,7 +2943,11 @@
         </is>
       </c>
       <c r="C72" s="142" t="n"/>
-      <c r="D72" s="35" t="n"/>
+      <c r="D72" s="35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="35" t="n"/>
@@ -2980,9 +3000,17 @@
           <t>E-6.1</t>
         </is>
       </c>
-      <c r="B80" s="139" t="n"/>
+      <c r="B80" s="139" t="inlineStr">
+        <is>
+          <t>Verificar comportamiento al reanudar la aplicación desde segundo plano</t>
+        </is>
+      </c>
       <c r="C80" s="140" t="n"/>
-      <c r="D80" s="36" t="n"/>
+      <c r="D80" s="36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="13.8" customHeight="1">
       <c r="A81" s="35" t="inlineStr">
@@ -2990,9 +3018,17 @@
           <t>E-6.2</t>
         </is>
       </c>
-      <c r="B81" s="141" t="n"/>
+      <c r="B81" s="141" t="inlineStr">
+        <is>
+          <t>Verificar que el sistema maneje adecuadamente la pérdida temporal de conexión</t>
+        </is>
+      </c>
       <c r="C81" s="142" t="n"/>
-      <c r="D81" s="36" t="n"/>
+      <c r="D81" s="36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="13.8" customHeight="1">
       <c r="A82" s="35" t="inlineStr">
@@ -3000,9 +3036,17 @@
           <t>E-6.3</t>
         </is>
       </c>
-      <c r="B82" s="94" t="n"/>
+      <c r="B82" s="94" t="inlineStr">
+        <is>
+          <t>Verificar compatibilidad con impresión de tickets de soporte físico</t>
+        </is>
+      </c>
       <c r="C82" s="95" t="n"/>
-      <c r="D82" s="36" t="n"/>
+      <c r="D82" s="36" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="13.8" customHeight="1">
       <c r="A83" s="35" t="n"/>
@@ -3334,7 +3378,7 @@
       <c r="C8" s="146" t="n"/>
       <c r="D8" s="126" t="inlineStr">
         <is>
-          <t>Marco Tassara Carrasco</t>
+          <t>Marco Tassara Carrasco / Miguel Arredondo Vargas</t>
         </is>
       </c>
       <c r="E8" s="145" t="n"/>
@@ -5709,6 +5753,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>La barra de navegación renderiza correctamente las opciones según el rol del usuario.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="25" t="n"/>
@@ -5825,6 +5874,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>La campana dibuja el número correcto de alertas pendientes de forma dinámica.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="25" t="n"/>
@@ -5941,6 +5995,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>El modal de pago valida que los campos de tarjeta no estén vacíos y requiere adjunto.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="25" t="n"/>
@@ -6055,6 +6114,11 @@
       <c r="J82" s="25" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>La página de Login valida que los campos no estén vacíos y despliega los mensajes de error locales.</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7197,6 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="L17:L19"/>
     <mergeCell ref="L60:L61"/>
-    <mergeCell ref="E46:E48"/>
     <mergeCell ref="D34:D36"/>
     <mergeCell ref="B43:B45"/>
     <mergeCell ref="N60:N61"/>
@@ -7248,6 +7311,7 @@
     <mergeCell ref="C46:C48"/>
     <mergeCell ref="A46:A48"/>
     <mergeCell ref="M28:M30"/>
+    <mergeCell ref="E46:E48"/>
     <mergeCell ref="K46:K48"/>
     <mergeCell ref="N17:N19"/>
   </mergeCells>

</xml_diff>

<commit_message>
test(android): agregar 5 pruebas para CrearOfertaViewModel, comentar tests de Login y actualizar documentacion de QA
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -2727,8 +2727,8 @@
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B77:C77"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B77:C77"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B86:C86"/>
@@ -2792,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X163"/>
+  <dimension ref="A1:X199"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.109375" customWidth="1" style="106" min="1" max="1"/>
@@ -6728,15 +6728,57 @@
       <c r="I125" s="77" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="77" t="n"/>
-      <c r="B126" s="77" t="n"/>
-      <c r="C126" s="77" t="n"/>
-      <c r="D126" s="77" t="n"/>
-      <c r="E126" s="77" t="n"/>
-      <c r="F126" s="77" t="n"/>
-      <c r="G126" s="77" t="n"/>
-      <c r="H126" s="77" t="n"/>
-      <c r="I126" s="77" t="n"/>
+      <c r="A126" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="B126" s="77" t="inlineStr">
+        <is>
+          <t>Publicar oferta</t>
+        </is>
+      </c>
+      <c r="C126" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D126" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E126" s="77" t="n">
+        <v>37</v>
+      </c>
+      <c r="F126" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de inicialización de publicación (CrearOfertaViewModel)</t>
+        </is>
+      </c>
+      <c r="G126" s="77" t="inlineStr">
+        <is>
+          <t>1. Inicializar el CrearOfertaViewModel con dependencias mockeadas en JUnit.</t>
+        </is>
+      </c>
+      <c r="H126" s="77" t="inlineStr">
+        <is>
+          <t>CrearOfertaViewModel inicializado, estado inicial vacío.</t>
+        </is>
+      </c>
+      <c r="I126" s="77" t="inlineStr">
+        <is>
+          <t>El estado inicial del formulario está completamente vacío con valores por defecto.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Se verifica con éxito que el formulario inicie limpio y sin datos precargados.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="77" t="n"/>
@@ -6772,15 +6814,57 @@
       <c r="I129" s="77" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="77" t="n"/>
-      <c r="B130" s="77" t="n"/>
-      <c r="C130" s="77" t="n"/>
-      <c r="D130" s="77" t="n"/>
-      <c r="E130" s="77" t="n"/>
-      <c r="F130" s="77" t="n"/>
-      <c r="G130" s="77" t="n"/>
-      <c r="H130" s="77" t="n"/>
-      <c r="I130" s="77" t="n"/>
+      <c r="A130" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="B130" s="77" t="inlineStr">
+        <is>
+          <t>Publicar oferta</t>
+        </is>
+      </c>
+      <c r="C130" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D130" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E130" s="77" t="n">
+        <v>38</v>
+      </c>
+      <c r="F130" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de modificación de campos de publicación</t>
+        </is>
+      </c>
+      <c r="G130" s="77" t="inlineStr">
+        <is>
+          <t>1. Simular ingreso de título, descripción, ubicación, categoría, remuneración y fechas.</t>
+        </is>
+      </c>
+      <c r="H130" s="77" t="inlineStr">
+        <is>
+          <t>Campos de la oferta de trabajo para Conserje.</t>
+        </is>
+      </c>
+      <c r="I130" s="77" t="inlineStr">
+        <is>
+          <t>El estado interno del ViewModel se actualiza correctamente reflejando las entradas del usuario.</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>Se comprueba la correcta persistencia en memoria de las modificaciones en el formulario.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="77" t="n"/>
@@ -6816,15 +6900,58 @@
       <c r="I133" s="77" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="77" t="n"/>
-      <c r="B134" s="77" t="n"/>
-      <c r="C134" s="77" t="n"/>
-      <c r="D134" s="77" t="n"/>
-      <c r="E134" s="77" t="n"/>
-      <c r="F134" s="77" t="n"/>
-      <c r="G134" s="77" t="n"/>
-      <c r="H134" s="77" t="n"/>
-      <c r="I134" s="77" t="n"/>
+      <c r="A134" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="B134" s="77" t="inlineStr">
+        <is>
+          <t>Publicar oferta</t>
+        </is>
+      </c>
+      <c r="C134" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D134" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E134" s="77" t="n">
+        <v>39</v>
+      </c>
+      <c r="F134" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de campos obligatorios faltantes en publicación</t>
+        </is>
+      </c>
+      <c r="G134" s="77" t="inlineStr">
+        <is>
+          <t>1. Rellenar campos omitiendo la fecha de inicio.
+2. Ejecutar submit().</t>
+        </is>
+      </c>
+      <c r="H134" s="77" t="inlineStr">
+        <is>
+          <t>Oferta incompleta (falta fechaInicio).</t>
+        </is>
+      </c>
+      <c r="I134" s="77" t="inlineStr">
+        <is>
+          <t>Se interrumpe la ejecución de publicación y se asigna el mensaje de error local indicando completar campos obligatorios.</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>Se valida el control local del formulario antes de interactuar con la API.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="77" t="n"/>
@@ -6860,15 +6987,59 @@
       <c r="I137" s="77" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="77" t="n"/>
-      <c r="B138" s="77" t="n"/>
-      <c r="C138" s="77" t="n"/>
-      <c r="D138" s="77" t="n"/>
-      <c r="E138" s="77" t="n"/>
-      <c r="F138" s="77" t="n"/>
-      <c r="G138" s="77" t="n"/>
-      <c r="H138" s="77" t="n"/>
-      <c r="I138" s="77" t="n"/>
+      <c r="A138" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="B138" s="77" t="inlineStr">
+        <is>
+          <t>Publicar oferta</t>
+        </is>
+      </c>
+      <c r="C138" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D138" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E138" s="77" t="n">
+        <v>40</v>
+      </c>
+      <c r="F138" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de publicación exitosa de oferta laboral</t>
+        </is>
+      </c>
+      <c r="G138" s="77" t="inlineStr">
+        <is>
+          <t>1. Cargar campos válidos.
+2. Mockear sesión de empresa y respuesta de éxito en JobsApi.create.
+3. Ejecutar submit().</t>
+        </is>
+      </c>
+      <c r="H138" s="77" t="inlineStr">
+        <is>
+          <t>CrearJobOfferRequest con datos válidos de Conserje.</t>
+        </is>
+      </c>
+      <c r="I138" s="77" t="inlineStr">
+        <is>
+          <t>Se llama a jobsApi.create y el estado final success queda en true sin errores.</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Se valida el flujo feliz y la llamada exitosa a la API de ofertas.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="77" t="n"/>
@@ -6904,15 +7075,59 @@
       <c r="I141" s="77" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="77" t="n"/>
-      <c r="B142" s="77" t="n"/>
-      <c r="C142" s="77" t="n"/>
-      <c r="D142" s="77" t="n"/>
-      <c r="E142" s="77" t="n"/>
-      <c r="F142" s="77" t="n"/>
-      <c r="G142" s="77" t="n"/>
-      <c r="H142" s="77" t="n"/>
-      <c r="I142" s="77" t="n"/>
+      <c r="A142" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="B142" s="77" t="inlineStr">
+        <is>
+          <t>Publicar oferta</t>
+        </is>
+      </c>
+      <c r="C142" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D142" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E142" s="77" t="n">
+        <v>41</v>
+      </c>
+      <c r="F142" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de fallo en la API al publicar oferta</t>
+        </is>
+      </c>
+      <c r="G142" s="77" t="inlineStr">
+        <is>
+          <t>1. Cargar campos válidos.
+2. Mockear una excepción IOException en la llamada a JobsApi.create.
+3. Ejecutar submit().</t>
+        </is>
+      </c>
+      <c r="H142" s="77" t="inlineStr">
+        <is>
+          <t>CrearJobOfferRequest válido, error del servidor simulado.</t>
+        </is>
+      </c>
+      <c r="I142" s="77" t="inlineStr">
+        <is>
+          <t>La excepción es capturada, el estado final success queda en false y se despliega el mensaje de error de la API.</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Se comprueba el manejo y despliegue del error de red/servidor ante fallos de publicación.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="77" t="n"/>
@@ -7145,6 +7360,42 @@
       <c r="H163" s="77" t="n"/>
       <c r="I163" s="77" t="n"/>
     </row>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <autoFilter ref="A12:N13"/>
   <mergeCells count="282">
@@ -7312,7 +7563,6 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="L17:L19"/>
     <mergeCell ref="L60:L61"/>
-    <mergeCell ref="E46:E48"/>
     <mergeCell ref="D34:D36"/>
     <mergeCell ref="B43:B45"/>
     <mergeCell ref="N60:N61"/>
@@ -7428,6 +7678,7 @@
     <mergeCell ref="M46:M48"/>
     <mergeCell ref="A46:A48"/>
     <mergeCell ref="L67:L68"/>
+    <mergeCell ref="E46:E48"/>
     <mergeCell ref="K46:K48"/>
     <mergeCell ref="N17:N19"/>
   </mergeCells>
@@ -7500,7 +7751,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -7510,7 +7761,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Sincronizar documentacion QA y agregar pruebas unitarias ErrorMapper y OfferDetailViewModel (CP-42 al CP-51)
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -2792,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X199"/>
+  <dimension ref="A1:X249"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.109375" customWidth="1" style="106" min="1" max="1"/>
@@ -7163,15 +7163,57 @@
       <c r="I145" s="77" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="77" t="n"/>
-      <c r="B146" s="77" t="n"/>
-      <c r="C146" s="77" t="n"/>
-      <c r="D146" s="77" t="n"/>
-      <c r="E146" s="77" t="n"/>
-      <c r="F146" s="77" t="n"/>
-      <c r="G146" s="77" t="n"/>
-      <c r="H146" s="77" t="n"/>
-      <c r="I146" s="77" t="n"/>
+      <c r="A146" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B146" s="77" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C146" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D146" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E146" s="77" t="n">
+        <v>42</v>
+      </c>
+      <c r="F146" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de mapeo de SocketTimeoutException (ErrorMapper)</t>
+        </is>
+      </c>
+      <c r="G146" s="77" t="inlineStr">
+        <is>
+          <t>1. Invocar ErrorMapper.map pasando una instancia de SocketTimeoutException.</t>
+        </is>
+      </c>
+      <c r="H146" s="77" t="inlineStr">
+        <is>
+          <t>SocketTimeoutException simulada.</t>
+        </is>
+      </c>
+      <c r="I146" s="77" t="inlineStr">
+        <is>
+          <t>El mapeador retorna ApiError.Timeout con el mensaje 'La solicitud demoró demasiado'.</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Se valida el mapeo correcto de errores de tiempo de respuesta de red.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="77" t="n"/>
@@ -7207,15 +7249,57 @@
       <c r="I149" s="77" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="77" t="n"/>
-      <c r="B150" s="77" t="n"/>
-      <c r="C150" s="77" t="n"/>
-      <c r="D150" s="77" t="n"/>
-      <c r="E150" s="77" t="n"/>
-      <c r="F150" s="77" t="n"/>
-      <c r="G150" s="77" t="n"/>
-      <c r="H150" s="77" t="n"/>
-      <c r="I150" s="77" t="n"/>
+      <c r="A150" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B150" s="77" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C150" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D150" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E150" s="77" t="n">
+        <v>43</v>
+      </c>
+      <c r="F150" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de mapeo de IOException (ErrorMapper)</t>
+        </is>
+      </c>
+      <c r="G150" s="77" t="inlineStr">
+        <is>
+          <t>1. Invocar ErrorMapper.map pasando una instancia de IOException.</t>
+        </is>
+      </c>
+      <c r="H150" s="77" t="inlineStr">
+        <is>
+          <t>IOException simulada.</t>
+        </is>
+      </c>
+      <c r="I150" s="77" t="inlineStr">
+        <is>
+          <t>El mapeador retorna ApiError.NoConnection con el mensaje 'Sin conexión a internet'.</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Se valida el mapeo correcto de desconexiones o fallas de red físicas.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="77" t="n"/>
@@ -7251,15 +7335,57 @@
       <c r="I153" s="77" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="77" t="n"/>
-      <c r="B154" s="77" t="n"/>
-      <c r="C154" s="77" t="n"/>
-      <c r="D154" s="77" t="n"/>
-      <c r="E154" s="77" t="n"/>
-      <c r="F154" s="77" t="n"/>
-      <c r="G154" s="77" t="n"/>
-      <c r="H154" s="77" t="n"/>
-      <c r="I154" s="77" t="n"/>
+      <c r="A154" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B154" s="77" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C154" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D154" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E154" s="77" t="n">
+        <v>44</v>
+      </c>
+      <c r="F154" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de mapeo de excepciones genéricas (ErrorMapper)</t>
+        </is>
+      </c>
+      <c r="G154" s="77" t="inlineStr">
+        <is>
+          <t>1. Invocar ErrorMapper.map con una RuntimeException genérica.</t>
+        </is>
+      </c>
+      <c r="H154" s="77" t="inlineStr">
+        <is>
+          <t>RuntimeException simulada con mensaje de error.</t>
+        </is>
+      </c>
+      <c r="I154" s="77" t="inlineStr">
+        <is>
+          <t>El mapeador retorna ApiError.Unknown conservando el mensaje original de la excepción.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Se comprueba la robustez del mapeador ante excepciones no controladas.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="77" t="n"/>
@@ -7295,15 +7421,58 @@
       <c r="I157" s="77" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="77" t="n"/>
-      <c r="B158" s="77" t="n"/>
-      <c r="C158" s="77" t="n"/>
-      <c r="D158" s="77" t="n"/>
-      <c r="E158" s="77" t="n"/>
-      <c r="F158" s="77" t="n"/>
-      <c r="G158" s="77" t="n"/>
-      <c r="H158" s="77" t="n"/>
-      <c r="I158" s="77" t="n"/>
+      <c r="A158" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B158" s="77" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C158" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D158" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E158" s="77" t="n">
+        <v>45</v>
+      </c>
+      <c r="F158" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de mapeo de error HTTP 401 (ErrorMapper)</t>
+        </is>
+      </c>
+      <c r="G158" s="77" t="inlineStr">
+        <is>
+          <t>1. Mockear HttpException con código 401.
+2. Invocar ErrorMapper.map.</t>
+        </is>
+      </c>
+      <c r="H158" s="77" t="inlineStr">
+        <is>
+          <t>HttpException 401 mockeada.</t>
+        </is>
+      </c>
+      <c r="I158" s="77" t="inlineStr">
+        <is>
+          <t>El mapeador retorna ApiError.Unauthorized con el mensaje de sesión expirada.</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Se verifica el mapeo correcto de errores de autorización del token JWT.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="77" t="n"/>
@@ -7339,15 +7508,58 @@
       <c r="I161" s="77" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="77" t="n"/>
-      <c r="B162" s="77" t="n"/>
-      <c r="C162" s="77" t="n"/>
-      <c r="D162" s="77" t="n"/>
-      <c r="E162" s="77" t="n"/>
-      <c r="F162" s="77" t="n"/>
-      <c r="G162" s="77" t="n"/>
-      <c r="H162" s="77" t="n"/>
-      <c r="I162" s="77" t="n"/>
+      <c r="A162" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B162" s="77" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C162" s="77" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D162" s="77" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E162" s="77" t="n">
+        <v>46</v>
+      </c>
+      <c r="F162" s="77" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de mapeo de error HTTP 404 (ErrorMapper)</t>
+        </is>
+      </c>
+      <c r="G162" s="77" t="inlineStr">
+        <is>
+          <t>1. Mockear HttpException con código 404.
+2. Invocar ErrorMapper.map.</t>
+        </is>
+      </c>
+      <c r="H162" s="77" t="inlineStr">
+        <is>
+          <t>HttpException 404 mockeada.</t>
+        </is>
+      </c>
+      <c r="I162" s="77" t="inlineStr">
+        <is>
+          <t>El mapeador retorna ApiError.NotFound con el mensaje de recurso no encontrado.</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>Se comprueba el mapeo de recursos inexistentes solicitados a la API.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="77" t="n"/>
@@ -7362,23 +7574,286 @@
     </row>
     <row r="164"/>
     <row r="165"/>
-    <row r="166"/>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>5</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Postular a oferta</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>47</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de carga de detalles de oferta (OfferDetailViewModel)</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>1. Inicializar el OfferDetailViewModel con el ID 101.
+2. Mockear respuesta de éxito en jobsRepository.getOffer(101).</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>OfferDetailViewModel con ID 101, respuesta exitosa mockeada.</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>El estado del ViewModel almacena los datos de la oferta y isLoading se establece en false.</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>Se valida la carga correcta de la vista de detalles al ingresar desde el feed.</t>
+        </is>
+      </c>
+    </row>
     <row r="167"/>
     <row r="168"/>
     <row r="169"/>
-    <row r="170"/>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>5</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Postular a oferta</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>48</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de fallo al cargar la oferta</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>1. Mockear excepción de red en jobsRepository.getOffer(102).
+2. Inicializar el ViewModel con ID 102.</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>ID de oferta 102, excepción de red mockeada.</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Se cancela la carga, isLoading queda en false y el mensaje de error de red se mapea correctamente en errorMessage.</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>Se comprueba la gestión del flujo fallido de carga de oferta.</t>
+        </is>
+      </c>
+    </row>
     <row r="171"/>
     <row r="172"/>
     <row r="173"/>
-    <row r="174"/>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>5</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Postular a oferta</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>49</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de postulación exitosa a oferta</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>1. Invocar submitApplication con un mensaje de presentación en el ViewModel.</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Mensaje: 'Me interesa el turno'.</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Se llama a applicationsRepository.apply(), isApplying queda en false, y no se presentan errores.</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>Se verifica el envío correcto del mensaje de postulación al repositorio.</t>
+        </is>
+      </c>
+    </row>
     <row r="175"/>
     <row r="176"/>
     <row r="177"/>
-    <row r="178"/>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>5</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Postular a oferta</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>50</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de postulación fallida por error del servidor</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>1. Mockear excepción IOException en applicationsRepository.apply().
+2. Invocar submitApplication.</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Excepción de red simulada.</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>isApplying queda en false y applyError se actualiza con la descripción de error de conexión traducida.</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>Se comprueba la tolerancia a fallos en el envío de postulaciones.</t>
+        </is>
+      </c>
+    </row>
     <row r="179"/>
     <row r="180"/>
     <row r="181"/>
-    <row r="182"/>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>5</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Postular a oferta</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>51</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de cancelación exitosa de postulación</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>1. Invocar cancelPostulation con el ID de postulación 999.</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>ID de postulación: 999.</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Se llama a cancelApplication y se actualizan los estados correctamente sin errores.</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>Se comprueba la anulación correcta del flujo de postulación por parte del usuario.</t>
+        </is>
+      </c>
+    </row>
     <row r="183"/>
     <row r="184"/>
     <row r="185"/>
@@ -7396,6 +7871,56 @@
     <row r="197"/>
     <row r="198"/>
     <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
   </sheetData>
   <autoFilter ref="A12:N13"/>
   <mergeCells count="282">
@@ -7751,7 +8276,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -7761,7 +8286,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Agregar pruebas unitarias para NotificationsViewModel (CP-52 al CP-56) y Sincronizar documentacion QA
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -2792,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X249"/>
+  <dimension ref="A1:X299"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.109375" customWidth="1" style="106" min="1" max="1"/>
@@ -7857,23 +7857,290 @@
     <row r="183"/>
     <row r="184"/>
     <row r="185"/>
-    <row r="186"/>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>8</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>52</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de estado inicial por defecto (NotificationsViewModel)</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>1. Inicializar el NotificationsViewModel.
+2. Comprobar que la lista de notificaciones esté vacía, el estado de conexión sea false y el conteo de no leídas sea 0.</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>ViewModel con dependencias mockeadas.</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>notifications es vacío, isConnected es false y unreadCount es 0.</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Se valida la inicialización correcta del estado del ViewModel sin notificaciones activas.</t>
+        </is>
+      </c>
+    </row>
     <row r="187"/>
     <row r="188"/>
     <row r="189"/>
-    <row r="190"/>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>8</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>53</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de cálculo de notificaciones no leídas (NotificationsViewModel)</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>1. Simular una lista de notificaciones con 2 no leídas y 1 leída.
+2. Actualizar el StateFlow del repositorio.
+3. Comprobar que unreadCount se actualice a 2.</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Lista de 3 notificaciones (2 con isRead = false, 1 con isRead = true).</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>El valor expuesto por unreadCount es exactamente 2.</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>Se comprueba el cálculo reactivo correcto del contador de notificaciones no leídas.</t>
+        </is>
+      </c>
+    </row>
     <row r="191"/>
     <row r="192"/>
     <row r="193"/>
-    <row r="194"/>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>8</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>54</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de marcar notificación como leída (NotificationsViewModel)</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>1. Invocar markAsRead("alerta_99") en el ViewModel.
+2. Verificar que se invoque markAsRead("alerta_99") en el repositorio.</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>ID de alerta: "alerta_99".</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Se invoca a notificationRepository.markAsRead("alerta_99") exactamente 1 vez.</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>Se valida la delegación correcta al repositorio para marcar como leída.</t>
+        </is>
+      </c>
+    </row>
     <row r="195"/>
     <row r="196"/>
     <row r="197"/>
-    <row r="198"/>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>8</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>55</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de limpiar notificaciones no leídas (NotificationsViewModel)</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>1. Cargar lista de notificaciones con pendientes.
+2. Invocar clearUnread().
+3. Verificar llamadas a markAsRead en el repositorio solo para las no leídas.</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Lista con notificaciones leídas y no leídas.</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Se invoca a markAsRead() en el repositorio solo para los IDs de notificaciones no leídas.</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Se comprueba la limpieza y marcado masivo de alertas pendientes.</t>
+        </is>
+      </c>
+    </row>
     <row r="199"/>
     <row r="200"/>
     <row r="201"/>
-    <row r="202"/>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>8</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>android-app</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>56</v>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Prueba unitaria de limpiar todas las notificaciones (NotificationsViewModel)</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>1. Invocar clearAll() en el ViewModel.
+2. Verificar que se llame a clearAll() en el repositorio.</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>ViewModel inicializado.</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Se invoca a notificationRepository.clearAll() exactamente 1 vez.</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>Se valida la eliminación y limpieza total del historial de notificaciones.</t>
+        </is>
+      </c>
+    </row>
     <row r="203"/>
     <row r="204"/>
     <row r="205"/>
@@ -7921,6 +8188,56 @@
     <row r="247"/>
     <row r="248"/>
     <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
   </sheetData>
   <autoFilter ref="A12:N13"/>
   <mergeCells count="282">
@@ -8276,7 +8593,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -8286,7 +8603,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Pruebas unitarias frontend RegisterPage y actualizacion de plan de pruebas en Word y Excel (CP-62 a CP-64)
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -2789,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X299"/>
+  <dimension ref="A1:X349"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.109375" customWidth="1" style="112" min="1" max="1"/>
@@ -9276,15 +9276,178 @@
     <row r="223" customFormat="1" s="112"/>
     <row r="224" customFormat="1" s="112"/>
     <row r="225" customFormat="1" s="112"/>
-    <row r="226" customFormat="1" s="112"/>
+    <row r="226" customFormat="1" s="112">
+      <c r="A226" t="n">
+        <v>1</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Registrar usuario</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>62</v>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Prueba de validación de fortaleza de contraseña (RegisterPage)</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>1. Cargar campos válidos en el formulario de registro.
+2. Escribir contraseña débil (sin mayúsculas o números).
+3. Hacer click en Crear Cuenta.</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Contraseña débil: 'weakpass'</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>El formulario se bloquea y muestra el mensaje de error: 'Mínimo 8 caracteres, 1 mayúscula y 1 número'.</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>Se verifica la correcta validación local de contraseñas seguras antes del envío.</t>
+        </is>
+      </c>
+    </row>
     <row r="227" customFormat="1" s="112"/>
     <row r="228" customFormat="1" s="112"/>
     <row r="229" customFormat="1" s="112"/>
-    <row r="230" customFormat="1" s="112"/>
+    <row r="230" customFormat="1" s="112">
+      <c r="A230" t="n">
+        <v>1</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Registrar usuario</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>63</v>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Prueba de coincidencia de contraseñas (RegisterPage)</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>1. Cargar campos válidos.
+2. Escribir contraseñas diferentes en los campos Contraseña y Confirmar.
+3. Hacer click en Crear Cuenta.</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>Contraseña: 'Secured123', Confirmar: 'Different123'.</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>El formulario se bloquea y muestra el mensaje de error: 'Las contraseñas no coinciden'.</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>Se comprueba la validación local de igualdad de claves.</t>
+        </is>
+      </c>
+    </row>
     <row r="231" customFormat="1" s="112"/>
     <row r="232" customFormat="1" s="112"/>
     <row r="233" customFormat="1" s="112"/>
-    <row r="234" customFormat="1" s="112"/>
+    <row r="234" customFormat="1" s="112">
+      <c r="A234" t="n">
+        <v>1</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Registrar usuario</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>64</v>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Prueba de flujo completo de registro exitoso tras aceptar términos (RegisterPage)</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>1. Cargar todos los campos válidos de registro.
+2. Hacer click en Crear Cuenta.
+3. En el modal de términos, hacer click en Aceptar y Registrarse.
+4. Mockear respuesta exitosa de authApi.register.</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Usuario: Juan Perez, RUT: 12345678-9, Email: juan@test.com, Teléfono: +56 912345678.</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Se realiza el registro en la API, se almacena el token JWT y los datos de sesión en localStorage, y se redirige a /trabajador/perfil.</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>Se valida el flujo exitoso completo del registro de nuevos trabajadores y su persistencia de sesión.</t>
+        </is>
+      </c>
+    </row>
     <row r="235" customFormat="1" s="112"/>
     <row r="236" customFormat="1" s="112"/>
     <row r="237" customFormat="1" s="112"/>
@@ -9350,6 +9513,56 @@
     <row r="297" customFormat="1" s="112"/>
     <row r="298" customFormat="1" s="112"/>
     <row r="299" customFormat="1" s="112"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
   </sheetData>
   <autoFilter ref="A12:N13"/>
   <mergeCells count="282">
@@ -9518,7 +9731,6 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="L17:L19"/>
     <mergeCell ref="L60:L61"/>
-    <mergeCell ref="E46:E48"/>
     <mergeCell ref="D34:D36"/>
     <mergeCell ref="B43:B45"/>
     <mergeCell ref="N60:N61"/>
@@ -9633,6 +9845,7 @@
     <mergeCell ref="C46:C48"/>
     <mergeCell ref="A46:A48"/>
     <mergeCell ref="M28:M30"/>
+    <mergeCell ref="E46:E48"/>
     <mergeCell ref="K46:K48"/>
     <mergeCell ref="N17:N19"/>
   </mergeCells>
@@ -9705,7 +9918,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -9715,7 +9928,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Pruebas unitarias backend JwtService y WebpayController y actualizacion de plan de pruebas en Word y Excel (CP-65 a CP-72)
</commit_message>
<xml_diff>
--- a/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Unidad #3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -9451,35 +9451,463 @@
     <row r="235" customFormat="1" s="112"/>
     <row r="236" customFormat="1" s="112"/>
     <row r="237" customFormat="1" s="112"/>
-    <row r="238" customFormat="1" s="112"/>
+    <row r="238" customFormat="1" s="112">
+      <c r="A238" t="n">
+        <v>2</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>65</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Prueba de generación exitosa de JWT (JwtService)</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>1. Invocar generateToken pasando un subject y tiempo de expiración.
+2. Comprobar que la respuesta no sea nula y tenga el formato JWT correcto.</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Subject: 'user@test.com', Expiración: 3600 segundos</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Se genera un string JWT compacto no vacío con tres secciones (header, payload y firma) separadas por puntos.</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>Se valida que el token se firme correctamente con la clave secreta HMAC-SHA.</t>
+        </is>
+      </c>
+    </row>
     <row r="239" customFormat="1" s="112"/>
     <row r="240" customFormat="1" s="112"/>
     <row r="241" customFormat="1" s="112"/>
-    <row r="242" customFormat="1" s="112"/>
+    <row r="242" customFormat="1" s="112">
+      <c r="A242" t="n">
+        <v>2</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>66</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Prueba de lectura correcta de Claims (JwtService)</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>1. Generar un token JWT válido con un subject y expiración específicos.
+2. Decodificar el token con parseClaims.
+3. Comprobar que los claims coincidan.</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Subject: 'test-user-id-999', Expiración: 1800 segundos</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>El método parseClaims extrae exitosamente el subject y el tiempo de expiración correcto del token decodificado.</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>Se verifica que la lectura de claims coincida con los datos del token generado.</t>
+        </is>
+      </c>
+    </row>
     <row r="243" customFormat="1" s="112"/>
     <row r="244" customFormat="1" s="112"/>
     <row r="245" customFormat="1" s="112"/>
-    <row r="246" customFormat="1" s="112"/>
+    <row r="246" customFormat="1" s="112">
+      <c r="A246" t="n">
+        <v>2</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>67</v>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Prueba de detección de alteración/tampering en token (JwtService)</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>1. Generar un token JWT válido.
+2. Alterar un caracter del token para invalidar su firma.
+3. Invocar parseClaims con el token alterado.</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>Token alterado con firma corrupta.</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>El método parseClaims detecta la alteración de la firma y lanza una excepción de tipo SignatureException.</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>Se comprueba que el sistema no acepte tokens cuya firma ha sido manipulada.</t>
+        </is>
+      </c>
+    </row>
     <row r="247" customFormat="1" s="112"/>
     <row r="248" customFormat="1" s="112"/>
     <row r="249" customFormat="1" s="112"/>
-    <row r="250" customFormat="1" s="112"/>
+    <row r="250" customFormat="1" s="112">
+      <c r="A250" t="n">
+        <v>2</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>68</v>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Prueba de control de expiración de token (JwtService)</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>1. Generar un token JWT con tiempo de expiración en el pasado.
+2. Invocar parseClaims con el token expirado.</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Expiración: -10 segundos.</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>El método parseClaims lanza una excepción de tipo ExpiredJwtException indicando que el token ya no es válido.</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>Se verifica el rechazo automático de tokens cuya fecha de expiración ha vencido.</t>
+        </is>
+      </c>
+    </row>
     <row r="251" customFormat="1" s="112"/>
     <row r="252" customFormat="1" s="112"/>
     <row r="253" customFormat="1" s="112"/>
-    <row r="254" customFormat="1" s="112"/>
+    <row r="254" customFormat="1" s="112">
+      <c r="A254" t="n">
+        <v>10</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>69</v>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Prueba de validación de parámetros faltantes al iniciar pago (WebpayController)</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>1. Enviar una petición POST a /profiles/webpay/init omitiendo el parámetro amount.
+2. Comprobar la respuesta HTTP.</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Payload JSON sin campo 'amount'.</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Retorna HTTP 400 Bad Request y un JSON indicando que los campos userId, amount y returnUrl son requeridos.</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>Se verifica la validación de campos obligatorios en el controlador de Webpay.</t>
+        </is>
+      </c>
+    </row>
     <row r="255" customFormat="1" s="112"/>
     <row r="256" customFormat="1" s="112"/>
     <row r="257" customFormat="1" s="112"/>
-    <row r="258" customFormat="1" s="112"/>
+    <row r="258" customFormat="1" s="112">
+      <c r="A258" t="n">
+        <v>10</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>70</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Prueba de inicialización exitosa de transacción (WebpayController)</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>1. Enviar una petición POST a /profiles/webpay/init con todos los parámetros correctos.
+2. Mockear respuesta exitosa del servicio Webpay.
+3. Comprobar la respuesta HTTP.</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>userId: 'user-123', amount: 10000, returnUrl: 'http://localhost/return'.</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Retorna HTTP 200 OK y una respuesta JSON que contiene el token de transacción y la URL de redirección.</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>Se valida el flujo correcto para iniciar la pasarela de pago en el controlador.</t>
+        </is>
+      </c>
+    </row>
     <row r="259" customFormat="1" s="112"/>
     <row r="260" customFormat="1" s="112"/>
     <row r="261" customFormat="1" s="112"/>
-    <row r="262" customFormat="1" s="112"/>
+    <row r="262" customFormat="1" s="112">
+      <c r="A262" t="n">
+        <v>10</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>71</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Prueba de validación de token faltante al confirmar pago (WebpayController)</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>1. Enviar una petición POST a /profiles/webpay/confirm con payload vacío o sin el token.
+2. Comprobar la respuesta HTTP.</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Payload JSON vacío.</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Retorna HTTP 400 Bad Request y un mensaje de error indicando que el token es requerido.</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>Se verifica la validación del token obligatorio para la confirmación de pago.</t>
+        </is>
+      </c>
+    </row>
     <row r="263" customFormat="1" s="112"/>
     <row r="264" customFormat="1" s="112"/>
     <row r="265" customFormat="1" s="112"/>
-    <row r="266" customFormat="1" s="112"/>
+    <row r="266" customFormat="1" s="112">
+      <c r="A266" t="n">
+        <v>10</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Prueba Unitarias</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>72</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Prueba de confirmación exitosa de transacción (WebpayController)</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>1. Enviar una petición POST a /profiles/webpay/confirm con un token válido.
+2. Mockear respuesta exitosa del servicio confirmando la transacción.
+3. Comprobar la respuesta HTTP.</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>token: 'real-token-123'.</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Retorna HTTP 200 OK y una respuesta JSON indicando que el estado de la transacción es AUTHORIZED.</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>Se valida el procesamiento exitoso de confirmación de pago del controlador.</t>
+        </is>
+      </c>
+    </row>
     <row r="267" customFormat="1" s="112"/>
     <row r="268" customFormat="1" s="112"/>
     <row r="269" customFormat="1" s="112"/>
@@ -9918,7 +10346,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
@@ -9928,7 +10356,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13">

</xml_diff>